<commit_message>
Update as of March 14, 2025 at 10:51 AM
</commit_message>
<xml_diff>
--- a/res/excel/kg_bases/kg_data.xlsx
+++ b/res/excel/kg_bases/kg_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aldri\OneDrive\Desktop\WLP_Automation-v5\res\excel\kg_bases\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aldri\OneDrive\Desktop\Nikka System\WLP_Automation-v7\res\excel\kg_bases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B8625DC-F85E-4F26-A55C-7598D72E50FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90BB807B-B5C2-48DA-8DC7-A67E81D0D049}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{4CF32C47-9F9A-4D90-BC6A-E165977FEF81}"/>
   </bookViews>
@@ -219,7 +219,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.000000000"/>
+    <numFmt numFmtId="173" formatCode="0.000"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
@@ -563,7 +563,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -625,9 +625,6 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -694,9 +691,6 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -736,7 +730,58 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -754,59 +799,35 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="173" fontId="5" fillId="6" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="6" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="173" fontId="5" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="173" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="173" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="173" fontId="5" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="173" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="173" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="173" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -826,9 +847,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -866,7 +887,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -972,7 +993,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1114,7 +1135,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1156,84 +1177,84 @@
     <col min="39" max="39" width="21.44140625" bestFit="1" customWidth="1"/>
     <col min="40" max="40" width="12.44140625" customWidth="1"/>
     <col min="41" max="41" width="12.5546875" customWidth="1"/>
-    <col min="42" max="42" width="12.5546875" style="57" customWidth="1"/>
-    <col min="43" max="47" width="8.88671875" style="57"/>
+    <col min="42" max="42" width="12.5546875" style="55" customWidth="1"/>
+    <col min="43" max="47" width="8.88671875" style="55"/>
     <col min="48" max="48" width="9.33203125" bestFit="1" customWidth="1"/>
     <col min="53" max="53" width="9.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:53" s="1" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4"/>
-      <c r="B1" s="58" t="s">
+      <c r="B1" s="73" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="60"/>
-      <c r="D1" s="60"/>
-      <c r="E1" s="60"/>
-      <c r="F1" s="60"/>
-      <c r="G1" s="60"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="58" t="s">
+      <c r="C1" s="75"/>
+      <c r="D1" s="75"/>
+      <c r="E1" s="75"/>
+      <c r="F1" s="75"/>
+      <c r="G1" s="75"/>
+      <c r="H1" s="76"/>
+      <c r="I1" s="73" t="s">
         <v>6</v>
       </c>
-      <c r="J1" s="76"/>
-      <c r="K1" s="58" t="s">
+      <c r="J1" s="79"/>
+      <c r="K1" s="73" t="s">
         <v>7</v>
       </c>
-      <c r="L1" s="60"/>
-      <c r="M1" s="76"/>
-      <c r="N1" s="76"/>
-      <c r="O1" s="61"/>
-      <c r="P1" s="59" t="s">
+      <c r="L1" s="75"/>
+      <c r="M1" s="79"/>
+      <c r="N1" s="79"/>
+      <c r="O1" s="76"/>
+      <c r="P1" s="74" t="s">
         <v>8</v>
       </c>
-      <c r="Q1" s="60"/>
-      <c r="R1" s="61"/>
-      <c r="S1" s="58" t="s">
+      <c r="Q1" s="75"/>
+      <c r="R1" s="76"/>
+      <c r="S1" s="73" t="s">
         <v>9</v>
       </c>
-      <c r="T1" s="59"/>
-      <c r="U1" s="59"/>
-      <c r="V1" s="59"/>
-      <c r="W1" s="59"/>
-      <c r="X1" s="59"/>
-      <c r="Y1" s="59"/>
-      <c r="Z1" s="59"/>
-      <c r="AA1" s="59"/>
-      <c r="AB1" s="59"/>
-      <c r="AC1" s="60"/>
-      <c r="AD1" s="58" t="s">
+      <c r="T1" s="74"/>
+      <c r="U1" s="74"/>
+      <c r="V1" s="74"/>
+      <c r="W1" s="74"/>
+      <c r="X1" s="74"/>
+      <c r="Y1" s="74"/>
+      <c r="Z1" s="74"/>
+      <c r="AA1" s="74"/>
+      <c r="AB1" s="74"/>
+      <c r="AC1" s="75"/>
+      <c r="AD1" s="73" t="s">
         <v>10</v>
       </c>
-      <c r="AE1" s="60"/>
-      <c r="AF1" s="60"/>
-      <c r="AG1" s="60"/>
-      <c r="AH1" s="60"/>
-      <c r="AI1" s="60"/>
-      <c r="AJ1" s="60"/>
-      <c r="AK1" s="60"/>
-      <c r="AL1" s="60"/>
-      <c r="AM1" s="61"/>
-      <c r="AN1" s="62" t="s">
+      <c r="AE1" s="75"/>
+      <c r="AF1" s="75"/>
+      <c r="AG1" s="75"/>
+      <c r="AH1" s="75"/>
+      <c r="AI1" s="75"/>
+      <c r="AJ1" s="75"/>
+      <c r="AK1" s="75"/>
+      <c r="AL1" s="75"/>
+      <c r="AM1" s="76"/>
+      <c r="AN1" s="77" t="s">
         <v>33</v>
       </c>
-      <c r="AO1" s="63"/>
-      <c r="AP1" s="71" t="s">
+      <c r="AO1" s="78"/>
+      <c r="AP1" s="69" t="s">
         <v>51</v>
       </c>
-      <c r="AQ1" s="72"/>
-      <c r="AR1" s="72"/>
-      <c r="AS1" s="72"/>
-      <c r="AT1" s="72"/>
-      <c r="AU1" s="72"/>
-      <c r="AV1" s="75"/>
-      <c r="AW1" s="71" t="s">
+      <c r="AQ1" s="70"/>
+      <c r="AR1" s="70"/>
+      <c r="AS1" s="70"/>
+      <c r="AT1" s="70"/>
+      <c r="AU1" s="70"/>
+      <c r="AV1" s="71"/>
+      <c r="AW1" s="69" t="s">
         <v>52</v>
       </c>
-      <c r="AX1" s="72"/>
-      <c r="AY1" s="72"/>
-      <c r="AZ1" s="72"/>
-      <c r="BA1" s="73"/>
+      <c r="AX1" s="70"/>
+      <c r="AY1" s="70"/>
+      <c r="AZ1" s="70"/>
+      <c r="BA1" s="72"/>
     </row>
     <row r="2" spans="1:53" s="3" customFormat="1" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5"/>
@@ -1264,10 +1285,10 @@
       <c r="J2" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="K2" s="80" t="s">
+      <c r="K2" s="67" t="s">
         <v>60</v>
       </c>
-      <c r="L2" s="81" t="s">
+      <c r="L2" s="68" t="s">
         <v>61</v>
       </c>
       <c r="M2" s="2" t="s">
@@ -1354,40 +1375,40 @@
       <c r="AN2" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="AO2" s="64" t="s">
+      <c r="AO2" s="56" t="s">
         <v>35</v>
       </c>
-      <c r="AP2" s="74" t="s">
+      <c r="AP2" s="63" t="s">
         <v>45</v>
       </c>
-      <c r="AQ2" s="70" t="s">
+      <c r="AQ2" s="62" t="s">
         <v>46</v>
       </c>
-      <c r="AR2" s="70" t="s">
+      <c r="AR2" s="62" t="s">
         <v>47</v>
       </c>
-      <c r="AS2" s="70" t="s">
+      <c r="AS2" s="62" t="s">
         <v>48</v>
       </c>
-      <c r="AT2" s="70" t="s">
+      <c r="AT2" s="62" t="s">
         <v>49</v>
       </c>
-      <c r="AU2" s="70" t="s">
+      <c r="AU2" s="62" t="s">
         <v>50</v>
       </c>
-      <c r="AV2" s="64" t="s">
+      <c r="AV2" s="56" t="s">
         <v>15</v>
       </c>
-      <c r="AW2" s="74" t="s">
+      <c r="AW2" s="63" t="s">
         <v>53</v>
       </c>
-      <c r="AX2" s="70" t="s">
+      <c r="AX2" s="62" t="s">
         <v>54</v>
       </c>
-      <c r="AY2" s="70" t="s">
+      <c r="AY2" s="62" t="s">
         <v>55</v>
       </c>
-      <c r="AZ2" s="70" t="s">
+      <c r="AZ2" s="62" t="s">
         <v>56</v>
       </c>
       <c r="BA2" s="9" t="s">
@@ -1408,7 +1429,7 @@
         <v>1.35</v>
       </c>
       <c r="I3" s="14"/>
-      <c r="J3" s="65">
+      <c r="J3" s="57">
         <v>5.4249999999999998</v>
       </c>
       <c r="K3" s="11">
@@ -1422,7 +1443,7 @@
         <v>22.41</v>
       </c>
       <c r="O3" s="13"/>
-      <c r="P3" s="52"/>
+      <c r="P3" s="50"/>
       <c r="Q3" s="16">
         <v>5.8</v>
       </c>
@@ -1430,20 +1451,20 @@
         <v>12.09</v>
       </c>
       <c r="S3" s="14"/>
-      <c r="T3" s="52"/>
-      <c r="U3" s="52"/>
-      <c r="V3" s="52"/>
-      <c r="W3" s="52"/>
-      <c r="X3" s="52"/>
-      <c r="Y3" s="52"/>
-      <c r="Z3" s="52"/>
-      <c r="AA3" s="52"/>
-      <c r="AB3" s="52"/>
+      <c r="T3" s="50"/>
+      <c r="U3" s="50"/>
+      <c r="V3" s="50"/>
+      <c r="W3" s="50"/>
+      <c r="X3" s="50"/>
+      <c r="Y3" s="50"/>
+      <c r="Z3" s="50"/>
+      <c r="AA3" s="50"/>
+      <c r="AB3" s="50"/>
       <c r="AC3" s="16"/>
       <c r="AD3" s="14"/>
       <c r="AE3" s="16"/>
       <c r="AF3" s="16"/>
-      <c r="AG3" s="16">
+      <c r="AG3" s="87">
         <v>0.3125</v>
       </c>
       <c r="AH3" s="16"/>
@@ -1453,7 +1474,7 @@
       <c r="AL3" s="16"/>
       <c r="AM3" s="15"/>
       <c r="AN3" s="14"/>
-      <c r="AO3" s="65"/>
+      <c r="AO3" s="57"/>
       <c r="AP3" s="11"/>
       <c r="AQ3" s="12"/>
       <c r="AR3" s="12"/>
@@ -1462,7 +1483,7 @@
       <c r="AU3" s="12">
         <v>2.38</v>
       </c>
-      <c r="AV3" s="65"/>
+      <c r="AV3" s="57"/>
       <c r="AW3" s="14"/>
       <c r="AX3" s="16"/>
       <c r="AY3" s="16"/>
@@ -1471,23 +1492,23 @@
         <v>3.25</v>
       </c>
     </row>
-    <row r="4" spans="1:53" s="26" customFormat="1" ht="22.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:53" s="25" customFormat="1" ht="22.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="18" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="19"/>
       <c r="C4" s="20"/>
-      <c r="D4" s="21">
+      <c r="D4" s="83">
         <v>6.0055180999999999E-2</v>
       </c>
       <c r="E4" s="20"/>
       <c r="F4" s="20"/>
       <c r="G4" s="20"/>
-      <c r="H4" s="22">
+      <c r="H4" s="21">
         <v>2.395</v>
       </c>
-      <c r="I4" s="23"/>
-      <c r="J4" s="66">
+      <c r="I4" s="22"/>
+      <c r="J4" s="58">
         <v>7.61</v>
       </c>
       <c r="K4" s="19">
@@ -1502,386 +1523,386 @@
       <c r="N4" s="20">
         <v>10.71</v>
       </c>
-      <c r="O4" s="22"/>
-      <c r="P4" s="53"/>
-      <c r="Q4" s="25"/>
-      <c r="R4" s="24">
+      <c r="O4" s="21"/>
+      <c r="P4" s="51"/>
+      <c r="Q4" s="24"/>
+      <c r="R4" s="23">
         <v>2.0550000000000002</v>
       </c>
-      <c r="S4" s="23">
+      <c r="S4" s="22">
         <v>2.5</v>
       </c>
-      <c r="T4" s="53">
+      <c r="T4" s="51">
         <v>1.69</v>
       </c>
-      <c r="U4" s="53"/>
-      <c r="V4" s="53"/>
-      <c r="W4" s="53"/>
-      <c r="X4" s="53"/>
-      <c r="Y4" s="53">
+      <c r="U4" s="51"/>
+      <c r="V4" s="51"/>
+      <c r="W4" s="51"/>
+      <c r="X4" s="51"/>
+      <c r="Y4" s="51">
         <v>0.92</v>
       </c>
-      <c r="Z4" s="53"/>
-      <c r="AA4" s="53"/>
-      <c r="AB4" s="53"/>
-      <c r="AC4" s="25"/>
-      <c r="AD4" s="23">
+      <c r="Z4" s="51"/>
+      <c r="AA4" s="51"/>
+      <c r="AB4" s="51"/>
+      <c r="AC4" s="24"/>
+      <c r="AD4" s="22">
         <v>3.25</v>
       </c>
-      <c r="AE4" s="25"/>
-      <c r="AF4" s="25"/>
-      <c r="AG4" s="25"/>
-      <c r="AH4" s="25">
+      <c r="AE4" s="24"/>
+      <c r="AF4" s="24"/>
+      <c r="AG4" s="24"/>
+      <c r="AH4" s="24">
         <v>11</v>
       </c>
-      <c r="AI4" s="25">
+      <c r="AI4" s="24">
         <v>9.1999999999999993</v>
       </c>
-      <c r="AJ4" s="25">
+      <c r="AJ4" s="24">
         <v>1</v>
       </c>
-      <c r="AK4" s="25">
+      <c r="AK4" s="24">
         <v>1.6</v>
       </c>
-      <c r="AL4" s="25">
+      <c r="AL4" s="88">
         <v>1.6666666670000001</v>
       </c>
-      <c r="AM4" s="24">
+      <c r="AM4" s="23">
         <v>1.75</v>
       </c>
-      <c r="AN4" s="23"/>
-      <c r="AO4" s="66"/>
+      <c r="AN4" s="22"/>
+      <c r="AO4" s="58"/>
       <c r="AP4" s="19"/>
       <c r="AQ4" s="20"/>
       <c r="AR4" s="20"/>
       <c r="AS4" s="20"/>
       <c r="AT4" s="20"/>
       <c r="AU4" s="20"/>
-      <c r="AV4" s="66">
+      <c r="AV4" s="58">
         <v>0.3</v>
       </c>
-      <c r="AW4" s="23"/>
-      <c r="AX4" s="25"/>
-      <c r="AY4" s="25"/>
-      <c r="AZ4" s="25"/>
-      <c r="BA4" s="24">
+      <c r="AW4" s="22"/>
+      <c r="AX4" s="24"/>
+      <c r="AY4" s="24"/>
+      <c r="AZ4" s="24"/>
+      <c r="BA4" s="23">
         <v>4.38</v>
       </c>
     </row>
-    <row r="5" spans="1:53" s="34" customFormat="1" ht="22.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="27" t="s">
+    <row r="5" spans="1:53" s="33" customFormat="1" ht="22.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="28"/>
-      <c r="C5" s="29">
+      <c r="B5" s="27"/>
+      <c r="C5" s="28">
         <v>8.8000000000000007</v>
       </c>
-      <c r="D5" s="29">
+      <c r="D5" s="84">
         <v>6.0055180999999999E-2</v>
       </c>
-      <c r="E5" s="29">
+      <c r="E5" s="28">
         <v>4.8600000000000003</v>
       </c>
-      <c r="F5" s="29">
+      <c r="F5" s="28">
         <v>1.6</v>
       </c>
-      <c r="G5" s="29">
+      <c r="G5" s="84">
         <v>14.395161290000001</v>
       </c>
-      <c r="H5" s="30">
+      <c r="H5" s="29">
         <v>8.64</v>
       </c>
-      <c r="I5" s="28">
+      <c r="I5" s="27">
         <v>3.2</v>
       </c>
-      <c r="J5" s="77">
+      <c r="J5" s="64">
         <v>5.56</v>
       </c>
-      <c r="K5" s="28">
+      <c r="K5" s="27">
         <v>10.42</v>
       </c>
-      <c r="L5" s="29"/>
-      <c r="M5" s="29"/>
-      <c r="N5" s="29"/>
-      <c r="O5" s="30">
+      <c r="L5" s="28"/>
+      <c r="M5" s="28"/>
+      <c r="N5" s="28"/>
+      <c r="O5" s="29">
         <v>10.62</v>
       </c>
-      <c r="P5" s="54"/>
-      <c r="Q5" s="32"/>
-      <c r="R5" s="33">
+      <c r="P5" s="52"/>
+      <c r="Q5" s="31"/>
+      <c r="R5" s="32">
         <v>11.82</v>
       </c>
-      <c r="S5" s="31">
+      <c r="S5" s="30">
         <v>2.5</v>
       </c>
-      <c r="T5" s="54">
+      <c r="T5" s="52">
         <v>1.69</v>
       </c>
-      <c r="U5" s="54">
+      <c r="U5" s="52">
         <v>1.1599999999999999</v>
       </c>
-      <c r="V5" s="54">
+      <c r="V5" s="52">
         <v>1.83</v>
       </c>
-      <c r="W5" s="54">
+      <c r="W5" s="52">
         <v>3.29</v>
       </c>
-      <c r="X5" s="54"/>
-      <c r="Y5" s="54">
+      <c r="X5" s="52"/>
+      <c r="Y5" s="52">
         <v>0.92</v>
       </c>
-      <c r="Z5" s="54">
+      <c r="Z5" s="52">
         <v>3.02</v>
       </c>
-      <c r="AA5" s="54">
+      <c r="AA5" s="52">
         <v>1.7</v>
       </c>
-      <c r="AB5" s="54"/>
-      <c r="AC5" s="32"/>
-      <c r="AD5" s="31"/>
-      <c r="AE5" s="29">
+      <c r="AB5" s="52"/>
+      <c r="AC5" s="31"/>
+      <c r="AD5" s="30"/>
+      <c r="AE5" s="28">
         <v>1.1000000000000001</v>
       </c>
-      <c r="AF5" s="32">
+      <c r="AF5" s="86">
         <v>3.2266666669999999</v>
       </c>
-      <c r="AG5" s="32"/>
-      <c r="AH5" s="32"/>
-      <c r="AI5" s="32"/>
-      <c r="AJ5" s="32"/>
-      <c r="AK5" s="32"/>
-      <c r="AL5" s="32"/>
-      <c r="AM5" s="33"/>
-      <c r="AN5" s="31">
+      <c r="AG5" s="31"/>
+      <c r="AH5" s="31"/>
+      <c r="AI5" s="31"/>
+      <c r="AJ5" s="31"/>
+      <c r="AK5" s="31"/>
+      <c r="AL5" s="31"/>
+      <c r="AM5" s="32"/>
+      <c r="AN5" s="30">
         <v>15.07</v>
       </c>
-      <c r="AO5" s="67">
+      <c r="AO5" s="59">
         <v>16.87</v>
       </c>
-      <c r="AP5" s="28"/>
-      <c r="AQ5" s="29"/>
-      <c r="AR5" s="29"/>
-      <c r="AS5" s="29"/>
-      <c r="AT5" s="29"/>
-      <c r="AU5" s="29"/>
-      <c r="AV5" s="67">
+      <c r="AP5" s="27"/>
+      <c r="AQ5" s="28"/>
+      <c r="AR5" s="28"/>
+      <c r="AS5" s="28"/>
+      <c r="AT5" s="28"/>
+      <c r="AU5" s="28"/>
+      <c r="AV5" s="59">
         <v>17.440000000000001</v>
       </c>
-      <c r="AW5" s="31"/>
-      <c r="AX5" s="32"/>
-      <c r="AY5" s="32"/>
-      <c r="AZ5" s="32"/>
-      <c r="BA5" s="33">
+      <c r="AW5" s="30"/>
+      <c r="AX5" s="31"/>
+      <c r="AY5" s="31"/>
+      <c r="AZ5" s="31"/>
+      <c r="BA5" s="32">
         <v>22.21</v>
       </c>
     </row>
-    <row r="6" spans="1:53" s="42" customFormat="1" ht="22.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="35" t="s">
+    <row r="6" spans="1:53" s="41" customFormat="1" ht="22.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="36"/>
-      <c r="C6" s="37"/>
-      <c r="D6" s="37">
+      <c r="B6" s="35"/>
+      <c r="C6" s="36"/>
+      <c r="D6" s="85">
         <v>6.0055180999999999E-2</v>
       </c>
-      <c r="E6" s="37"/>
-      <c r="F6" s="37">
+      <c r="E6" s="36"/>
+      <c r="F6" s="36">
         <v>1.6</v>
       </c>
-      <c r="G6" s="37">
+      <c r="G6" s="85">
         <v>14.395161290000001</v>
       </c>
-      <c r="H6" s="38">
+      <c r="H6" s="37">
         <v>8.64</v>
       </c>
-      <c r="I6" s="39"/>
-      <c r="J6" s="78">
+      <c r="I6" s="38"/>
+      <c r="J6" s="65">
         <v>3.21</v>
       </c>
-      <c r="K6" s="36"/>
-      <c r="L6" s="37"/>
-      <c r="M6" s="37"/>
-      <c r="N6" s="37"/>
-      <c r="O6" s="38"/>
-      <c r="P6" s="55"/>
-      <c r="Q6" s="40"/>
-      <c r="R6" s="41">
+      <c r="K6" s="35"/>
+      <c r="L6" s="36"/>
+      <c r="M6" s="36"/>
+      <c r="N6" s="36"/>
+      <c r="O6" s="37"/>
+      <c r="P6" s="53"/>
+      <c r="Q6" s="39"/>
+      <c r="R6" s="40">
         <v>9.6</v>
       </c>
-      <c r="S6" s="39">
+      <c r="S6" s="38">
         <v>2.5</v>
       </c>
-      <c r="T6" s="55"/>
-      <c r="U6" s="55">
+      <c r="T6" s="53"/>
+      <c r="U6" s="53">
         <v>1.1599999999999999</v>
       </c>
-      <c r="V6" s="55">
+      <c r="V6" s="53">
         <v>1.83</v>
       </c>
-      <c r="W6" s="55"/>
-      <c r="X6" s="55">
+      <c r="W6" s="53"/>
+      <c r="X6" s="53">
         <v>1.1599999999999999</v>
       </c>
-      <c r="Y6" s="55">
+      <c r="Y6" s="53">
         <v>0.92</v>
       </c>
-      <c r="Z6" s="55">
+      <c r="Z6" s="53">
         <v>3.02</v>
       </c>
-      <c r="AA6" s="55">
+      <c r="AA6" s="53">
         <v>1.7</v>
       </c>
-      <c r="AB6" s="55">
+      <c r="AB6" s="53">
         <v>0.74</v>
       </c>
-      <c r="AC6" s="40">
+      <c r="AC6" s="39">
         <v>12.7</v>
       </c>
-      <c r="AD6" s="39"/>
-      <c r="AE6" s="40"/>
-      <c r="AF6" s="40"/>
-      <c r="AG6" s="40"/>
-      <c r="AH6" s="40"/>
-      <c r="AI6" s="40">
+      <c r="AD6" s="38"/>
+      <c r="AE6" s="39"/>
+      <c r="AF6" s="39"/>
+      <c r="AG6" s="39"/>
+      <c r="AH6" s="39"/>
+      <c r="AI6" s="39">
         <v>9.1999999999999993</v>
       </c>
-      <c r="AJ6" s="40"/>
-      <c r="AK6" s="40"/>
-      <c r="AL6" s="40"/>
-      <c r="AM6" s="41"/>
-      <c r="AN6" s="39">
+      <c r="AJ6" s="39"/>
+      <c r="AK6" s="39"/>
+      <c r="AL6" s="39"/>
+      <c r="AM6" s="40"/>
+      <c r="AN6" s="38">
         <v>15.07</v>
       </c>
-      <c r="AO6" s="68">
+      <c r="AO6" s="60">
         <v>16.87</v>
       </c>
-      <c r="AP6" s="36">
+      <c r="AP6" s="35">
         <v>10.07</v>
       </c>
-      <c r="AQ6" s="37"/>
-      <c r="AR6" s="37"/>
-      <c r="AS6" s="37"/>
-      <c r="AT6" s="37"/>
-      <c r="AU6" s="37"/>
-      <c r="AV6" s="68">
+      <c r="AQ6" s="36"/>
+      <c r="AR6" s="36"/>
+      <c r="AS6" s="36"/>
+      <c r="AT6" s="36"/>
+      <c r="AU6" s="36"/>
+      <c r="AV6" s="60">
         <v>3.2</v>
       </c>
-      <c r="AW6" s="39">
+      <c r="AW6" s="38">
         <v>3.92</v>
       </c>
-      <c r="AX6" s="40"/>
-      <c r="AY6" s="40"/>
-      <c r="AZ6" s="40"/>
-      <c r="BA6" s="41">
+      <c r="AX6" s="39"/>
+      <c r="AY6" s="39"/>
+      <c r="AZ6" s="39"/>
+      <c r="BA6" s="40">
         <v>3.92</v>
       </c>
     </row>
-    <row r="7" spans="1:53" s="51" customFormat="1" ht="22.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="43" t="s">
+    <row r="7" spans="1:53" s="49" customFormat="1" ht="22.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="42" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="44">
+      <c r="B7" s="82">
         <v>8.996975806</v>
       </c>
-      <c r="C7" s="45">
+      <c r="C7" s="43">
         <v>8.8000000000000007</v>
       </c>
-      <c r="D7" s="45">
+      <c r="D7" s="80">
         <v>6.0055180999999999E-2</v>
       </c>
-      <c r="E7" s="45">
+      <c r="E7" s="43">
         <v>4.8600000000000003</v>
       </c>
-      <c r="F7" s="45">
+      <c r="F7" s="43">
         <v>1.6</v>
       </c>
-      <c r="G7" s="45">
+      <c r="G7" s="80">
         <v>14.395161290000001</v>
       </c>
-      <c r="H7" s="46">
+      <c r="H7" s="81">
         <v>9.44</v>
       </c>
-      <c r="I7" s="47"/>
-      <c r="J7" s="79">
+      <c r="I7" s="45"/>
+      <c r="J7" s="66">
         <v>7.101</v>
       </c>
-      <c r="K7" s="48"/>
-      <c r="L7" s="45"/>
-      <c r="M7" s="45"/>
-      <c r="N7" s="45"/>
-      <c r="O7" s="46"/>
-      <c r="P7" s="56"/>
-      <c r="Q7" s="49"/>
-      <c r="R7" s="50"/>
-      <c r="S7" s="47"/>
-      <c r="T7" s="56"/>
-      <c r="U7" s="56"/>
-      <c r="V7" s="56"/>
-      <c r="W7" s="56"/>
-      <c r="X7" s="56"/>
-      <c r="Y7" s="56"/>
-      <c r="Z7" s="56"/>
-      <c r="AA7" s="56"/>
-      <c r="AB7" s="56"/>
-      <c r="AC7" s="49"/>
-      <c r="AD7" s="47"/>
-      <c r="AE7" s="49"/>
-      <c r="AF7" s="49"/>
-      <c r="AG7" s="49"/>
-      <c r="AH7" s="49"/>
-      <c r="AI7" s="49"/>
-      <c r="AJ7" s="49"/>
-      <c r="AK7" s="49"/>
-      <c r="AL7" s="49"/>
-      <c r="AM7" s="50"/>
-      <c r="AN7" s="47">
+      <c r="K7" s="46"/>
+      <c r="L7" s="43"/>
+      <c r="M7" s="43"/>
+      <c r="N7" s="43"/>
+      <c r="O7" s="44"/>
+      <c r="P7" s="54"/>
+      <c r="Q7" s="47"/>
+      <c r="R7" s="48"/>
+      <c r="S7" s="45"/>
+      <c r="T7" s="54"/>
+      <c r="U7" s="54"/>
+      <c r="V7" s="54"/>
+      <c r="W7" s="54"/>
+      <c r="X7" s="54"/>
+      <c r="Y7" s="54"/>
+      <c r="Z7" s="54"/>
+      <c r="AA7" s="54"/>
+      <c r="AB7" s="54"/>
+      <c r="AC7" s="47"/>
+      <c r="AD7" s="45"/>
+      <c r="AE7" s="47"/>
+      <c r="AF7" s="47"/>
+      <c r="AG7" s="47"/>
+      <c r="AH7" s="47"/>
+      <c r="AI7" s="47"/>
+      <c r="AJ7" s="47"/>
+      <c r="AK7" s="47"/>
+      <c r="AL7" s="47"/>
+      <c r="AM7" s="48"/>
+      <c r="AN7" s="45">
         <v>15.07</v>
       </c>
-      <c r="AO7" s="69">
+      <c r="AO7" s="61">
         <v>16.87</v>
       </c>
-      <c r="AP7" s="48"/>
-      <c r="AQ7" s="45">
+      <c r="AP7" s="46"/>
+      <c r="AQ7" s="43">
         <v>17.309999999999999</v>
       </c>
-      <c r="AR7" s="45">
+      <c r="AR7" s="43">
         <v>10.81</v>
       </c>
-      <c r="AS7" s="45">
+      <c r="AS7" s="43">
         <v>64.239999999999995</v>
       </c>
-      <c r="AT7" s="45">
+      <c r="AT7" s="43">
         <v>7.23</v>
       </c>
-      <c r="AU7" s="45"/>
-      <c r="AV7" s="69">
+      <c r="AU7" s="43"/>
+      <c r="AV7" s="61">
         <v>15.19</v>
       </c>
-      <c r="AW7" s="47"/>
-      <c r="AX7" s="49">
+      <c r="AW7" s="45"/>
+      <c r="AX7" s="47">
         <v>10.119999999999999</v>
       </c>
-      <c r="AY7" s="49">
+      <c r="AY7" s="47">
         <v>46.65</v>
       </c>
-      <c r="AZ7" s="49">
+      <c r="AZ7" s="47">
         <v>10.17</v>
       </c>
-      <c r="BA7" s="50">
+      <c r="BA7" s="48">
         <v>52.27</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="9">
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="I1:J1"/>
+    <mergeCell ref="K1:O1"/>
+    <mergeCell ref="P1:R1"/>
     <mergeCell ref="AP1:AV1"/>
     <mergeCell ref="AW1:BA1"/>
     <mergeCell ref="S1:AC1"/>
     <mergeCell ref="AD1:AM1"/>
     <mergeCell ref="AN1:AO1"/>
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="I1:J1"/>
-    <mergeCell ref="K1:O1"/>
-    <mergeCell ref="P1:R1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
@@ -1893,41 +1914,41 @@
   <dimension ref="A1:M1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="13" width="8.88671875" style="57"/>
+    <col min="1" max="13" width="8.88671875" style="55"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="55" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="57" t="s">
+      <c r="B1" s="55" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="57" t="s">
+      <c r="C1" s="55" t="s">
         <v>36</v>
       </c>
-      <c r="D1" s="57" t="s">
+      <c r="D1" s="55" t="s">
         <v>37</v>
       </c>
-      <c r="E1" s="57" t="s">
+      <c r="E1" s="55" t="s">
         <v>38</v>
       </c>
-      <c r="F1" s="57" t="s">
+      <c r="F1" s="55" t="s">
         <v>39</v>
       </c>
-      <c r="G1" s="57" t="s">
+      <c r="G1" s="55" t="s">
         <v>40</v>
       </c>
-      <c r="H1" s="57" t="s">
+      <c r="H1" s="55" t="s">
         <v>41</v>
       </c>
-      <c r="I1" s="57" t="s">
+      <c r="I1" s="55" t="s">
         <v>42</v>
       </c>
-      <c r="J1" s="57" t="s">
+      <c r="J1" s="55" t="s">
         <v>43</v>
       </c>
-      <c r="K1" s="57" t="s">
+      <c r="K1" s="55" t="s">
         <v>44</v>
       </c>
     </row>

</xml_diff>